<commit_message>
Status of Funds: fiscal month (1 = Oct) column, filter and CSV; spending trend (cumulative vs straight-line pace vs spend plan, monthly bars, % of TDP vs % of year); optional spend plan file + template; third List rows step; tests
</commit_message>
<xml_diff>
--- a/dashboards/finance/data/funding_sample.xlsx
+++ b/dashboards/finance/data/funding_sample.xlsx
@@ -125,8 +125,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingData" displayName="FundingData" ref="A1:F60" headerRowCount="1">
-  <autoFilter ref="A1:F60"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FundingData" displayName="FundingData" ref="A1:F61" headerRowCount="1">
+  <autoFilter ref="A1:F61"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Fiscal Year"/>
     <tableColumn id="2" name="Functional Area"/>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,10 +480,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1043600</v>
+        <v>958500</v>
       </c>
       <c r="E2" t="n">
-        <v>1043600</v>
+        <v>958500</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -506,10 +506,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>527000</v>
+        <v>405800</v>
       </c>
       <c r="E3" t="n">
-        <v>527000</v>
+        <v>405800</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -532,10 +532,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>848700</v>
+        <v>106600</v>
       </c>
       <c r="E4" t="n">
-        <v>848700</v>
+        <v>106600</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -549,19 +549,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>244G92YYUK</t>
+          <t>287G64ZRCW</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Recruiting Travel</t>
+          <t>School Pay</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>219400</v>
+        <v>3017400</v>
       </c>
       <c r="E5" t="n">
-        <v>219400</v>
+        <v>3017400</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -575,19 +575,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>287G64ZRCW</t>
+          <t>329G26BYSX</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>School Pay</t>
+          <t>Family Programs</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1330000</v>
+        <v>375700</v>
       </c>
       <c r="E6" t="n">
-        <v>1330000</v>
+        <v>375700</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -601,19 +601,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>329G26BYSX</t>
+          <t>364G63URSS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Family Programs</t>
+          <t>Armory Custodial</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>27600</v>
+        <v>119100</v>
       </c>
       <c r="E7" t="n">
-        <v>27600</v>
+        <v>119100</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -627,19 +627,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>357G54MNZS</t>
+          <t>401G44ABEW</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Vehicle Maintenance</t>
+          <t>Aviation Fuel</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>311500</v>
+        <v>507500</v>
       </c>
       <c r="E8" t="n">
-        <v>311500</v>
+        <v>507500</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -653,19 +653,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>364G63URSS</t>
+          <t>424G68DQYY</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Armory Custodial</t>
+          <t>Annual Training Pay</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>481800</v>
+        <v>772700</v>
       </c>
       <c r="E9" t="n">
-        <v>481800</v>
+        <v>772700</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -679,19 +679,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>401G44ABEW</t>
+          <t>472G69PCNU</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Aviation Fuel</t>
+          <t>IT Equipment</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>218300</v>
+        <v>31000</v>
       </c>
       <c r="E10" t="n">
-        <v>218300</v>
+        <v>31000</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -705,19 +705,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>424G68DQYY</t>
+          <t>479G22GZPE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Annual Training Pay</t>
+          <t>Bonuses &amp; Incentives</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>710200</v>
+        <v>443700</v>
       </c>
       <c r="E11" t="n">
-        <v>710200</v>
+        <v>443700</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -731,19 +731,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>472G69PCNU</t>
+          <t>539G70ERHD</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>IT Equipment</t>
+          <t>Safety Training</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1452700</v>
+        <v>379900</v>
       </c>
       <c r="E12" t="n">
-        <v>1452700</v>
+        <v>379900</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -757,19 +757,19 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>479G22GZPE</t>
+          <t>551G40AVCD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bonuses &amp; Incentives</t>
+          <t>Doctor Support</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>508900</v>
+        <v>298500</v>
       </c>
       <c r="E13" t="n">
-        <v>508900</v>
+        <v>298500</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -783,19 +783,19 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>539G70ERHD</t>
+          <t>560G11XRXL</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Safety Training</t>
+          <t>Range Operations</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>52000</v>
+        <v>262600</v>
       </c>
       <c r="E14" t="n">
-        <v>52000</v>
+        <v>262600</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -809,19 +809,19 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>551G40AVCD</t>
+          <t>577G75RPTX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Doctor Support</t>
+          <t>Drill Pay</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>465200</v>
+        <v>837300</v>
       </c>
       <c r="E15" t="n">
-        <v>465200</v>
+        <v>837300</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -835,19 +835,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>560G11XRXL</t>
+          <t>661G92SYRN</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Range Operations</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>162400</v>
+        <v>36000</v>
       </c>
       <c r="E16" t="n">
-        <v>162400</v>
+        <v>36000</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -861,19 +861,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>577G75RPTX</t>
+          <t>736G81PUTZ</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Drill Pay</t>
+          <t>Lawyers</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1174000</v>
+        <v>237800</v>
       </c>
       <c r="E17" t="n">
-        <v>1174000</v>
+        <v>237800</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -887,19 +887,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>661G92SYRN</t>
+          <t>790G70YTJT</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Environmental Compliance</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>41800</v>
+        <v>594700</v>
       </c>
       <c r="E18" t="n">
-        <v>41800</v>
+        <v>594700</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -913,19 +913,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>736G81PUTZ</t>
+          <t>840G53CTTK</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Lawyers</t>
+          <t>Facility Utilities</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>526100</v>
+        <v>121300</v>
       </c>
       <c r="E19" t="n">
-        <v>526100</v>
+        <v>121300</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
@@ -939,19 +939,19 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>790G70YTJT</t>
+          <t>922G76RMGJ</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Environmental Compliance</t>
+          <t>Medical Readiness</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>43300</v>
+        <v>451700</v>
       </c>
       <c r="E20" t="n">
-        <v>43300</v>
+        <v>451700</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -965,19 +965,19 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>840G53CTTK</t>
+          <t>988G24PSVR</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Facility Utilities</t>
+          <t>Schools Travel</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>439100</v>
+        <v>241200</v>
       </c>
       <c r="E21" t="n">
-        <v>439100</v>
+        <v>241200</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -986,27 +986,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>FY26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>922G76RMGJ</t>
+          <t>194G10QUTC</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Medical Readiness</t>
+          <t>Readiness Center Repair</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>104500</v>
+        <v>308100</v>
       </c>
       <c r="E22" t="n">
-        <v>104500</v>
+        <v>306800</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>6546.32</v>
       </c>
     </row>
     <row r="23">
@@ -1017,22 +1017,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>194G10QUTC</t>
+          <t>221G50SSWD</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Readiness Center Repair</t>
+          <t>Course Supplies</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>63200</v>
+        <v>1170600</v>
       </c>
       <c r="E23" t="n">
-        <v>59500</v>
+        <v>1058700</v>
       </c>
       <c r="F23" t="n">
-        <v>627.77</v>
+        <v>28347.67</v>
       </c>
     </row>
     <row r="24">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>221G50SSWD</t>
+          <t>223G89BTJX</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Course Supplies</t>
+          <t>Range Construction</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>571300</v>
+        <v>749300</v>
       </c>
       <c r="E24" t="n">
-        <v>524000</v>
+        <v>728200</v>
       </c>
       <c r="F24" t="n">
-        <v>29812.11</v>
+        <v>23159.57</v>
       </c>
     </row>
     <row r="25">
@@ -1069,22 +1069,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>223G89BTJX</t>
+          <t>244G92YYUK</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Range Construction</t>
+          <t>Recruiting Travel</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>814900</v>
+        <v>198800</v>
       </c>
       <c r="E25" t="n">
-        <v>768000</v>
+        <v>183900</v>
       </c>
       <c r="F25" t="n">
-        <v>26780.86</v>
+        <v>13838</v>
       </c>
     </row>
     <row r="26">
@@ -1095,22 +1095,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>244G92YYUK</t>
+          <t>287G64ZRCW</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Recruiting Travel</t>
+          <t>School Pay</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>559500</v>
+        <v>1460000</v>
       </c>
       <c r="E26" t="n">
-        <v>541100</v>
+        <v>1339100</v>
       </c>
       <c r="F26" t="n">
-        <v>16090.62</v>
+        <v>72533.71000000001</v>
       </c>
     </row>
     <row r="27">
@@ -1121,22 +1121,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>287G64ZRCW</t>
+          <t>329G26BYSX</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>School Pay</t>
+          <t>Family Programs</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>2942400</v>
+        <v>529000</v>
       </c>
       <c r="E27" t="n">
-        <v>2805000</v>
+        <v>521600</v>
       </c>
       <c r="F27" t="n">
-        <v>108176.69</v>
+        <v>33103.16</v>
       </c>
     </row>
     <row r="28">
@@ -1147,22 +1147,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>329G26BYSX</t>
+          <t>357G54MNZS</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Family Programs</t>
+          <t>Vehicle Maintenance</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>273800</v>
+        <v>133500</v>
       </c>
       <c r="E28" t="n">
-        <v>262500</v>
+        <v>131000</v>
       </c>
       <c r="F28" t="n">
-        <v>18776.16</v>
+        <v>7614.2</v>
       </c>
     </row>
     <row r="29">
@@ -1173,22 +1173,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>357G54MNZS</t>
+          <t>364G63URSS</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Vehicle Maintenance</t>
+          <t>Armory Custodial</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>264000</v>
+        <v>405600</v>
       </c>
       <c r="E29" t="n">
-        <v>252500</v>
+        <v>401000</v>
       </c>
       <c r="F29" t="n">
-        <v>5040.12</v>
+        <v>24822.95</v>
       </c>
     </row>
     <row r="30">
@@ -1199,22 +1199,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>364G63URSS</t>
+          <t>401G44ABEW</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Armory Custodial</t>
+          <t>Aviation Fuel</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>6800</v>
+        <v>83400</v>
       </c>
       <c r="E30" t="n">
-        <v>6300</v>
+        <v>82000</v>
       </c>
       <c r="F30" t="n">
-        <v>242.69</v>
+        <v>2804.19</v>
       </c>
     </row>
     <row r="31">
@@ -1225,22 +1225,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>401G44ABEW</t>
+          <t>424G68DQYY</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Aviation Fuel</t>
+          <t>Annual Training Pay</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>240900</v>
+        <v>281000</v>
       </c>
       <c r="E31" t="n">
-        <v>229200</v>
+        <v>258200</v>
       </c>
       <c r="F31" t="n">
-        <v>10491.98</v>
+        <v>8129.84</v>
       </c>
     </row>
     <row r="32">
@@ -1251,22 +1251,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>424G68DQYY</t>
+          <t>472G69PCNU</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Annual Training Pay</t>
+          <t>IT Equipment</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1046700</v>
+        <v>692000</v>
       </c>
       <c r="E32" t="n">
-        <v>1025200</v>
+        <v>672300</v>
       </c>
       <c r="F32" t="n">
-        <v>23294.14</v>
+        <v>43725.27</v>
       </c>
     </row>
     <row r="33">
@@ -1277,22 +1277,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>472G69PCNU</t>
+          <t>479G22GZPE</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IT Equipment</t>
+          <t>Bonuses &amp; Incentives</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>284100</v>
+        <v>1426000</v>
       </c>
       <c r="E33" t="n">
-        <v>269900</v>
+        <v>1401300</v>
       </c>
       <c r="F33" t="n">
-        <v>14932.6</v>
+        <v>113305.23</v>
       </c>
     </row>
     <row r="34">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>479G22GZPE</t>
+          <t>539G70ERHD</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bonuses &amp; Incentives</t>
+          <t>Safety Training</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>757000</v>
+        <v>595800</v>
       </c>
       <c r="E34" t="n">
-        <v>722300</v>
+        <v>579900</v>
       </c>
       <c r="F34" t="n">
-        <v>14941.18</v>
+        <v>29998.23</v>
       </c>
     </row>
     <row r="35">
@@ -1329,22 +1329,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>539G70ERHD</t>
+          <t>551G40AVCD</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Safety Training</t>
+          <t>Doctor Support</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>161600</v>
+        <v>83200</v>
       </c>
       <c r="E35" t="n">
-        <v>151800</v>
+        <v>77300</v>
       </c>
       <c r="F35" t="n">
-        <v>7842.98</v>
+        <v>4072.73</v>
       </c>
     </row>
     <row r="36">
@@ -1355,22 +1355,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>551G40AVCD</t>
+          <t>560G11XRXL</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Doctor Support</t>
+          <t>Range Operations</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>113000</v>
+        <v>678100</v>
       </c>
       <c r="E36" t="n">
-        <v>106400</v>
+        <v>642200</v>
       </c>
       <c r="F36" t="n">
-        <v>2831.36</v>
+        <v>7354.87</v>
       </c>
     </row>
     <row r="37">
@@ -1381,22 +1381,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>560G11XRXL</t>
+          <t>577G75RPTX</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Range Operations</t>
+          <t>Drill Pay</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>394600</v>
+        <v>486900</v>
       </c>
       <c r="E37" t="n">
-        <v>381700</v>
+        <v>470500</v>
       </c>
       <c r="F37" t="n">
-        <v>13500.26</v>
+        <v>7162.46</v>
       </c>
     </row>
     <row r="38">
@@ -1407,22 +1407,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>577G75RPTX</t>
+          <t>661G92SYRN</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Drill Pay</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1352200</v>
+        <v>370500</v>
       </c>
       <c r="E38" t="n">
-        <v>1229200</v>
+        <v>340800</v>
       </c>
       <c r="F38" t="n">
-        <v>59435.63</v>
+        <v>12527.76</v>
       </c>
     </row>
     <row r="39">
@@ -1433,22 +1433,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>661G92SYRN</t>
+          <t>736G81PUTZ</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Lawyers</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1159100</v>
+        <v>543600</v>
       </c>
       <c r="E39" t="n">
-        <v>1125800</v>
+        <v>513300</v>
       </c>
       <c r="F39" t="n">
-        <v>5881.66</v>
+        <v>29866.86</v>
       </c>
     </row>
     <row r="40">
@@ -1459,22 +1459,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>736G81PUTZ</t>
+          <t>790G70YTJT</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Lawyers</t>
+          <t>Environmental Compliance</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>368400</v>
+        <v>313100</v>
       </c>
       <c r="E40" t="n">
-        <v>352400</v>
+        <v>301400</v>
       </c>
       <c r="F40" t="n">
-        <v>13964.47</v>
+        <v>7942.09</v>
       </c>
     </row>
     <row r="41">
@@ -1485,22 +1485,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>790G70YTJT</t>
+          <t>840G53CTTK</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Environmental Compliance</t>
+          <t>Facility Utilities</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>423900</v>
+        <v>336900</v>
       </c>
       <c r="E41" t="n">
-        <v>382900</v>
+        <v>317000</v>
       </c>
       <c r="F41" t="n">
-        <v>18937.28</v>
+        <v>5257.94</v>
       </c>
     </row>
     <row r="42">
@@ -1511,22 +1511,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>840G53CTTK</t>
+          <t>922G76RMGJ</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Facility Utilities</t>
+          <t>Medical Readiness</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>122000</v>
+        <v>551500</v>
       </c>
       <c r="E42" t="n">
-        <v>110500</v>
+        <v>505800</v>
       </c>
       <c r="F42" t="n">
-        <v>6775.67</v>
+        <v>19154.05</v>
       </c>
     </row>
     <row r="43">
@@ -1537,48 +1537,48 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>922G76RMGJ</t>
+          <t>988G24PSVR</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Medical Readiness</t>
+          <t>Schools Travel</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>408500</v>
+        <v>510800</v>
       </c>
       <c r="E43" t="n">
-        <v>394300</v>
+        <v>487400</v>
       </c>
       <c r="F43" t="n">
-        <v>6476.35</v>
+        <v>16370.72</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>FY26</t>
+          <t>FY27</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>988G24PSVR</t>
+          <t>223G89BTJX</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Schools Travel</t>
+          <t>Range Construction</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>706100</v>
+        <v>186400</v>
       </c>
       <c r="E44" t="n">
-        <v>696300</v>
+        <v>26500</v>
       </c>
       <c r="F44" t="n">
-        <v>22806.97</v>
+        <v>9797.32</v>
       </c>
     </row>
     <row r="45">
@@ -1589,22 +1589,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>221G50SSWD</t>
+          <t>244G92YYUK</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Course Supplies</t>
+          <t>Recruiting Travel</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>56700</v>
+        <v>65900</v>
       </c>
       <c r="E45" t="n">
-        <v>10300</v>
+        <v>15700</v>
       </c>
       <c r="F45" t="n">
-        <v>402.85</v>
+        <v>1497.19</v>
       </c>
     </row>
     <row r="46">
@@ -1615,22 +1615,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>244G92YYUK</t>
+          <t>287G64ZRCW</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Recruiting Travel</t>
+          <t>School Pay</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>86100</v>
+        <v>253500</v>
       </c>
       <c r="E46" t="n">
-        <v>18300</v>
+        <v>48800</v>
       </c>
       <c r="F46" t="n">
-        <v>3466.84</v>
+        <v>2415.51</v>
       </c>
     </row>
     <row r="47">
@@ -1641,22 +1641,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>287G64ZRCW</t>
+          <t>329G26BYSX</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>School Pay</t>
+          <t>Family Programs</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>177500</v>
+        <v>22500</v>
       </c>
       <c r="E47" t="n">
-        <v>25300</v>
+        <v>4600</v>
       </c>
       <c r="F47" t="n">
-        <v>7970.92</v>
+        <v>1505.34</v>
       </c>
     </row>
     <row r="48">
@@ -1667,22 +1667,22 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>329G26BYSX</t>
+          <t>357G54MNZS</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Family Programs</t>
+          <t>Vehicle Maintenance</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>126900</v>
+        <v>29900</v>
       </c>
       <c r="E48" t="n">
-        <v>21700</v>
+        <v>6200</v>
       </c>
       <c r="F48" t="n">
-        <v>7289.22</v>
+        <v>1316.43</v>
       </c>
     </row>
     <row r="49">
@@ -1702,13 +1702,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>107900</v>
+        <v>65600</v>
       </c>
       <c r="E49" t="n">
-        <v>20100</v>
+        <v>14300</v>
       </c>
       <c r="F49" t="n">
-        <v>7790.26</v>
+        <v>3211.96</v>
       </c>
     </row>
     <row r="50">
@@ -1719,22 +1719,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>401G44ABEW</t>
+          <t>472G69PCNU</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Aviation Fuel</t>
+          <t>IT Equipment</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>48700</v>
+        <v>11600</v>
       </c>
       <c r="E50" t="n">
-        <v>5000</v>
+        <v>1600</v>
       </c>
       <c r="F50" t="n">
-        <v>2420.46</v>
+        <v>896.89</v>
       </c>
     </row>
     <row r="51">
@@ -1745,22 +1745,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>424G68DQYY</t>
+          <t>479G22GZPE</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Annual Training Pay</t>
+          <t>Bonuses &amp; Incentives</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>217700</v>
+        <v>5000</v>
       </c>
       <c r="E51" t="n">
-        <v>22600</v>
+        <v>1000</v>
       </c>
       <c r="F51" t="n">
-        <v>13971.09</v>
+        <v>337.57</v>
       </c>
     </row>
     <row r="52">
@@ -1771,22 +1771,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>472G69PCNU</t>
+          <t>539G70ERHD</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>IT Equipment</t>
+          <t>Safety Training</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>13300</v>
+        <v>75900</v>
       </c>
       <c r="E52" t="n">
-        <v>1600</v>
+        <v>17200</v>
       </c>
       <c r="F52" t="n">
-        <v>7.18</v>
+        <v>2048.89</v>
       </c>
     </row>
     <row r="53">
@@ -1797,22 +1797,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>479G22GZPE</t>
+          <t>551G40AVCD</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Bonuses &amp; Incentives</t>
+          <t>Doctor Support</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>119300</v>
+        <v>98500</v>
       </c>
       <c r="E53" t="n">
-        <v>14900</v>
+        <v>21500</v>
       </c>
       <c r="F53" t="n">
-        <v>1487.99</v>
+        <v>7347.71</v>
       </c>
     </row>
     <row r="54">
@@ -1823,22 +1823,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>551G40AVCD</t>
+          <t>577G75RPTX</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Doctor Support</t>
+          <t>Drill Pay</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>68800</v>
+        <v>342800</v>
       </c>
       <c r="E54" t="n">
-        <v>6900</v>
+        <v>80600</v>
       </c>
       <c r="F54" t="n">
-        <v>2580.39</v>
+        <v>5275.18</v>
       </c>
     </row>
     <row r="55">
@@ -1849,22 +1849,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>577G75RPTX</t>
+          <t>736G81PUTZ</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Drill Pay</t>
+          <t>Lawyers</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>69900</v>
+        <v>146700</v>
       </c>
       <c r="E55" t="n">
-        <v>10900</v>
+        <v>35900</v>
       </c>
       <c r="F55" t="n">
-        <v>5194.24</v>
+        <v>10157.69</v>
       </c>
     </row>
     <row r="56">
@@ -1875,22 +1875,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>661G92SYRN</t>
+          <t>790G70YTJT</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>Environmental Compliance</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5000</v>
+        <v>59300</v>
       </c>
       <c r="E56" t="n">
-        <v>700</v>
+        <v>6400</v>
       </c>
       <c r="F56" t="n">
-        <v>288.06</v>
+        <v>1637.31</v>
       </c>
     </row>
     <row r="57">
@@ -1910,13 +1910,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>74600</v>
+        <v>5000</v>
       </c>
       <c r="E57" t="n">
-        <v>11400</v>
+        <v>1100</v>
       </c>
       <c r="F57" t="n">
-        <v>3753.8</v>
+        <v>220.38</v>
       </c>
     </row>
     <row r="58">
@@ -1936,13 +1936,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>17000</v>
+        <v>268000</v>
       </c>
       <c r="E58" t="n">
-        <v>3000</v>
+        <v>57100</v>
       </c>
       <c r="F58" t="n">
-        <v>1356.83</v>
+        <v>4196.5</v>
       </c>
     </row>
     <row r="59">
@@ -1953,22 +1953,22 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>194G10QUTC</t>
+          <t>988G24PSVR</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Readiness Center Repair</t>
+          <t>Schools Travel</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>120000</v>
+        <v>218700</v>
       </c>
       <c r="E59" t="n">
-        <v>15000</v>
+        <v>38000</v>
       </c>
       <c r="F59" t="n">
-        <v>2500</v>
+        <v>11605.5</v>
       </c>
     </row>
     <row r="60">
@@ -1979,12 +1979,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>223G89BTJX</t>
+          <t>424G68DQYY</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Range Construction</t>
+          <t>Annual Training Pay</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -1994,6 +1994,32 @@
         <v>15000</v>
       </c>
       <c r="F60" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>194G10QUTC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Readiness Center Repair</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>120000</v>
+      </c>
+      <c r="E61" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F61" t="n">
         <v>2500</v>
       </c>
     </row>

</xml_diff>